<commit_message>
change system in practitionerrole e8e9ca88400787c8123cbb0b00f4f5db240c1db4
</commit_message>
<xml_diff>
--- a/main/ig/StructureDefinition-as-dp-practitionerrole.xlsx
+++ b/main/ig/StructureDefinition-as-dp-practitionerrole.xlsx
@@ -60,7 +60,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2024-06-03T16:22:01+00:00</t>
+    <t>2024-06-03T16:23:50+00:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -878,7 +878,7 @@
     <t>There are many sets  of identifiers.  To perform matching of two identifiers, we need to know what set we're dealing with. The system identifies a particular set of unique identifiers.</t>
   </si>
   <si>
-    <t>http://rpps.fr</t>
+    <t>https://rpps.esante.gouv.fr</t>
   </si>
   <si>
     <t>http://www.acme.com/identifiers/patient</t>
@@ -1012,7 +1012,7 @@
     <t>PractitionerRole.identifier:numeroAm.system</t>
   </si>
   <si>
-    <t>http://ameli.fr</t>
+    <t>https://adeli.esante.gouv.fr</t>
   </si>
   <si>
     <t>PractitionerRole.identifier:numeroAm.value</t>

</xml_diff>

<commit_message>
Revert "change system in practitionerrole"
This reverts commit e8e9ca88400787c8123cbb0b00f4f5db240c1db4. 72e1ef11919e57b01ce1488aa81c122b476bbedc
</commit_message>
<xml_diff>
--- a/main/ig/StructureDefinition-as-dp-practitionerrole.xlsx
+++ b/main/ig/StructureDefinition-as-dp-practitionerrole.xlsx
@@ -60,7 +60,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2024-06-03T16:23:50+00:00</t>
+    <t>2024-06-03T16:30:34+00:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -878,7 +878,7 @@
     <t>There are many sets  of identifiers.  To perform matching of two identifiers, we need to know what set we're dealing with. The system identifies a particular set of unique identifiers.</t>
   </si>
   <si>
-    <t>https://rpps.esante.gouv.fr</t>
+    <t>http://rpps.fr</t>
   </si>
   <si>
     <t>http://www.acme.com/identifiers/patient</t>
@@ -1012,7 +1012,7 @@
     <t>PractitionerRole.identifier:numeroAm.system</t>
   </si>
   <si>
-    <t>https://adeli.esante.gouv.fr</t>
+    <t>http://ameli.fr</t>
   </si>
   <si>
     <t>PractitionerRole.identifier:numeroAm.value</t>

</xml_diff>

<commit_message>
Change system pr (RPPS & ADELI) (#209)
* change system pr

* Update AsPractitionerRoleProfile.fsh 5c5b4a7cd32f6984541757aaf0d88cf65f505772
</commit_message>
<xml_diff>
--- a/main/ig/StructureDefinition-as-dp-practitionerrole.xlsx
+++ b/main/ig/StructureDefinition-as-dp-practitionerrole.xlsx
@@ -60,7 +60,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2024-06-03T16:30:34+00:00</t>
+    <t>2024-06-05T12:07:44+00:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -878,7 +878,7 @@
     <t>There are many sets  of identifiers.  To perform matching of two identifiers, we need to know what set we're dealing with. The system identifies a particular set of unique identifiers.</t>
   </si>
   <si>
-    <t>http://rpps.fr</t>
+    <t>https://rpps.esante.gouv.fr</t>
   </si>
   <si>
     <t>http://www.acme.com/identifiers/patient</t>
@@ -1012,7 +1012,7 @@
     <t>PractitionerRole.identifier:numeroAm.system</t>
   </si>
   <si>
-    <t>http://ameli.fr</t>
+    <t>https://www.ameli.fr</t>
   </si>
   <si>
     <t>PractitionerRole.identifier:numeroAm.value</t>

</xml_diff>